<commit_message>
#3 BOM updated with two resistors
</commit_message>
<xml_diff>
--- a/Design Files/Breakout_PCB_Board_Design/BOM/Client_BOM.xlsx
+++ b/Design Files/Breakout_PCB_Board_Design/BOM/Client_BOM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12330"/>
+    <workbookView windowWidth="19635" windowHeight="7650"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="59">
   <si>
     <t>Component list</t>
   </si>
@@ -130,6 +130,24 @@
     <t>XKB Connectivity</t>
   </si>
   <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>R1, R2</t>
+  </si>
+  <si>
+    <t>1/4 watt Resistor</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>DNP</t>
+  </si>
+  <si>
     <t>Switch</t>
   </si>
   <si>
@@ -146,9 +164,6 @@
   </si>
   <si>
     <t>Peripheral</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>Adafruit ESP32 Feather V2 w.FL Antenna - 8MB Flash + 2 MB PSRAM - STEMMA QT</t>
@@ -183,11 +198,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9">
   <numFmts count="5">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="176" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="179" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="180" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
   <fonts count="39">
     <font>
@@ -321,8 +336,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -684,7 +699,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -830,6 +845,19 @@
       <left style="medium">
         <color auto="1"/>
       </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
       <right/>
       <top/>
       <bottom style="medium">
@@ -877,6 +905,34 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -991,19 +1047,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1012,7 +1068,7 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1024,34 +1080,34 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="27" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1136,7 +1192,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1210,7 +1266,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="176" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1240,10 +1296,22 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1266,36 +1334,51 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -1412,7 +1495,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14325600" y="619760"/>
+          <a:off x="14325600" y="629285"/>
           <a:ext cx="1857375" cy="1104265"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1683,7 +1766,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
@@ -1698,7 +1781,7 @@
     <col min="11" max="11" width="29.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" ht="15.75" spans="1:11">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1707,9 +1790,9 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
     </row>
     <row r="2" ht="32.25" spans="1:11">
       <c r="A2" s="2"/>
@@ -1719,14 +1802,14 @@
         <v>0</v>
       </c>
       <c r="E2" s="7"/>
-      <c r="F2" s="61" t="s">
+      <c r="F2" s="70" t="s">
         <v>1</v>
       </c>
       <c r="G2" s="8"/>
       <c r="H2" s="9"/>
       <c r="I2" s="9"/>
       <c r="J2" s="9"/>
-      <c r="K2" s="56"/>
+      <c r="K2" s="60"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="2"/>
@@ -1736,14 +1819,14 @@
         <v>2</v>
       </c>
       <c r="E3" s="12"/>
-      <c r="F3" s="62" t="s">
+      <c r="F3" s="71" t="s">
         <v>3</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="14"/>
       <c r="I3" s="14"/>
       <c r="J3" s="14"/>
-      <c r="K3" s="57"/>
+      <c r="K3" s="61"/>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2"/>
@@ -1760,7 +1843,7 @@
       <c r="H4" s="17"/>
       <c r="I4" s="17"/>
       <c r="J4" s="17"/>
-      <c r="K4" s="58"/>
+      <c r="K4" s="62"/>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="2"/>
@@ -1770,14 +1853,14 @@
         <v>5</v>
       </c>
       <c r="E5" s="12"/>
-      <c r="F5" s="63" t="s">
+      <c r="F5" s="72" t="s">
         <v>6</v>
       </c>
       <c r="G5" s="19"/>
       <c r="H5" s="20"/>
       <c r="I5" s="20"/>
       <c r="J5" s="20"/>
-      <c r="K5" s="58"/>
+      <c r="K5" s="62"/>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="2"/>
@@ -1790,7 +1873,7 @@
       <c r="H6" s="20"/>
       <c r="I6" s="20"/>
       <c r="J6" s="20"/>
-      <c r="K6" s="58"/>
+      <c r="K6" s="62"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2"/>
@@ -1803,9 +1886,9 @@
       <c r="H7" s="29"/>
       <c r="I7" s="29"/>
       <c r="J7" s="29"/>
-      <c r="K7" s="58"/>
+      <c r="K7" s="62"/>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" ht="15.75" spans="1:11">
       <c r="A8" s="2"/>
       <c r="B8" s="30"/>
       <c r="C8" s="31"/>
@@ -1816,9 +1899,9 @@
       <c r="H8" s="29"/>
       <c r="I8" s="29"/>
       <c r="J8" s="29"/>
-      <c r="K8" s="58"/>
+      <c r="K8" s="62"/>
     </row>
-    <row r="9" ht="15.75" spans="1:11">
+    <row r="9" spans="1:11">
       <c r="A9" s="2"/>
       <c r="B9" s="34" t="s">
         <v>7</v>
@@ -1835,7 +1918,7 @@
       <c r="F9" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="35" t="s">
+      <c r="G9" s="34" t="s">
         <v>12</v>
       </c>
       <c r="H9" s="34" t="s">
@@ -1869,7 +1952,7 @@
       <c r="F10" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="39" t="s">
+      <c r="G10" s="38" t="s">
         <v>21</v>
       </c>
       <c r="H10" s="38" t="s">
@@ -1878,15 +1961,15 @@
       <c r="I10" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="38">
+      <c r="J10" s="63">
         <v>4</v>
       </c>
-      <c r="K10" s="38"/>
+      <c r="K10" s="64"/>
     </row>
     <row r="11" ht="48.75" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="36">
-        <f t="shared" ref="B11:B14" si="0">ROW(B11)-ROW($B$9)</f>
+        <f>ROW(B11)-ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="40" t="s">
@@ -1901,7 +1984,7 @@
       <c r="F11" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="42" t="s">
+      <c r="G11" s="41" t="s">
         <v>26</v>
       </c>
       <c r="H11" s="41" t="s">
@@ -1910,7 +1993,7 @@
       <c r="I11" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="J11" s="41">
+      <c r="J11" s="65">
         <v>2</v>
       </c>
       <c r="K11" s="41"/>
@@ -1918,7 +2001,7 @@
     <row r="12" ht="36.75" spans="1:11">
       <c r="A12" s="2"/>
       <c r="B12" s="36">
-        <f t="shared" si="0"/>
+        <f>ROW(B12)-ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="37" t="s">
@@ -1933,7 +2016,7 @@
       <c r="F12" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="G12" s="39" t="s">
+      <c r="G12" s="38" t="s">
         <v>31</v>
       </c>
       <c r="H12" s="38" t="s">
@@ -1942,7 +2025,7 @@
       <c r="I12" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="J12" s="38">
+      <c r="J12" s="63">
         <v>1</v>
       </c>
       <c r="K12" s="38"/>
@@ -1950,7 +2033,7 @@
     <row r="13" ht="60.75" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="36">
-        <f t="shared" si="0"/>
+        <f>ROW(B13)-ROW($B$9)</f>
         <v>4</v>
       </c>
       <c r="C13" s="40" t="s">
@@ -1965,7 +2048,7 @@
       <c r="F13" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G13" s="42" t="s">
+      <c r="G13" s="41" t="s">
         <v>36</v>
       </c>
       <c r="H13" s="41" t="s">
@@ -1974,213 +2057,246 @@
       <c r="I13" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="J13" s="41">
+      <c r="J13" s="65">
         <v>1</v>
       </c>
       <c r="K13" s="41"/>
     </row>
-    <row r="14" ht="24.75" spans="1:11">
+    <row r="14" ht="15.75" spans="1:11">
       <c r="A14" s="2"/>
       <c r="B14" s="36">
-        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="37" t="s">
+      <c r="C14" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="39" t="s">
+      <c r="E14" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="38" t="s">
+      <c r="F14" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="39" t="s">
-        <v>41</v>
+      <c r="G14" s="38" t="s">
+        <v>42</v>
       </c>
       <c r="H14" s="38" t="s">
         <v>42</v>
       </c>
       <c r="I14" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="J14" s="38">
+        <v>42</v>
+      </c>
+      <c r="J14" s="66">
         <v>2</v>
       </c>
-      <c r="K14" s="43"/>
+      <c r="K14" s="67" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="15" ht="24.75" spans="1:11">
       <c r="A15" s="2"/>
-      <c r="B15" s="44"/>
+      <c r="B15" s="36">
+        <f>ROW(B15)-ROW($B$9)</f>
+        <v>6</v>
+      </c>
       <c r="C15" s="37" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="41" t="s">
         <v>44</v>
       </c>
+      <c r="D15" s="46" t="s">
+        <v>45</v>
+      </c>
       <c r="E15" s="39" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="G15" s="39" t="s">
-        <v>44</v>
+        <v>47</v>
+      </c>
+      <c r="G15" s="38" t="s">
+        <v>47</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I15" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="J15" s="38">
+        <v>47</v>
+      </c>
+      <c r="J15" s="63">
         <v>2</v>
       </c>
-      <c r="K15" s="38"/>
+      <c r="K15" s="41"/>
     </row>
-    <row r="16" ht="15.75" spans="1:11">
+    <row r="16" ht="24.75" spans="1:11">
       <c r="A16" s="2"/>
-      <c r="B16" s="44"/>
+      <c r="B16" s="47"/>
       <c r="C16" s="37" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="38" t="s">
-        <v>44</v>
+        <v>49</v>
+      </c>
+      <c r="D16" s="41" t="s">
+        <v>42</v>
       </c>
       <c r="E16" s="39" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F16" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="G16" s="39" t="s">
-        <v>44</v>
+        <v>42</v>
+      </c>
+      <c r="G16" s="38" t="s">
+        <v>42</v>
       </c>
       <c r="H16" s="38" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="I16" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="J16" s="38">
+        <v>42</v>
+      </c>
+      <c r="J16" s="63">
         <v>2</v>
       </c>
-      <c r="K16" s="38"/>
+      <c r="K16" s="41"/>
     </row>
-    <row r="17" ht="24.75" spans="1:11">
+    <row r="17" ht="15.75" spans="1:11">
       <c r="A17" s="2"/>
-      <c r="B17" s="44"/>
+      <c r="B17" s="47"/>
       <c r="C17" s="37" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E17" s="39" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="G17" s="39" t="s">
-        <v>44</v>
+        <v>42</v>
+      </c>
+      <c r="G17" s="38" t="s">
+        <v>42</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I17" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="J17" s="38">
+        <v>42</v>
+      </c>
+      <c r="J17" s="63">
         <v>2</v>
       </c>
       <c r="K17" s="38"/>
     </row>
-    <row r="18" ht="15.75" spans="1:11">
+    <row r="18" ht="24.75" spans="1:11">
       <c r="A18" s="2"/>
-      <c r="B18" s="44"/>
+      <c r="B18" s="47"/>
       <c r="C18" s="37" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D18" s="38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E18" s="39" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F18" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="G18" s="39" t="s">
-        <v>44</v>
+        <v>42</v>
+      </c>
+      <c r="G18" s="38" t="s">
+        <v>42</v>
       </c>
       <c r="H18" s="38" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I18" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="J18" s="38">
-        <v>1</v>
+        <v>42</v>
+      </c>
+      <c r="J18" s="63">
+        <v>2</v>
       </c>
       <c r="K18" s="38"/>
     </row>
-    <row r="19" ht="15.75" spans="1:11">
+    <row r="19" spans="1:11">
       <c r="A19" s="2"/>
-      <c r="B19" s="44"/>
+      <c r="B19" s="47"/>
       <c r="C19" s="37" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E19" s="39" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="G19" s="39" t="s">
-        <v>44</v>
+        <v>42</v>
+      </c>
+      <c r="G19" s="38" t="s">
+        <v>42</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="I19" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="J19" s="38">
+        <v>42</v>
+      </c>
+      <c r="J19" s="63">
         <v>1</v>
       </c>
       <c r="K19" s="38"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="2"/>
-      <c r="B20" s="45"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="50"/>
-      <c r="H20" s="49"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="50"/>
-      <c r="K20" s="59"/>
+      <c r="B20" s="47"/>
+      <c r="C20" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>57</v>
+      </c>
+      <c r="F20" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="G20" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="H20" s="48" t="s">
+        <v>58</v>
+      </c>
+      <c r="I20" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="J20" s="63">
+        <v>1</v>
+      </c>
+      <c r="K20" s="48"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="2"/>
-      <c r="B21" s="51"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="54"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="50"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="53"/>
       <c r="G21" s="54"/>
-      <c r="H21" s="54"/>
+      <c r="H21" s="53"/>
       <c r="I21" s="54"/>
       <c r="J21" s="54"/>
-      <c r="K21" s="60"/>
+      <c r="K21" s="68"/>
+    </row>
+    <row r="22" ht="15.75" spans="1:11">
+      <c r="A22" s="2"/>
+      <c r="B22" s="55"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="57"/>
+      <c r="E22" s="58"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58"/>
+      <c r="H22" s="58"/>
+      <c r="I22" s="58"/>
+      <c r="J22" s="58"/>
+      <c r="K22" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>